<commit_message>
Fill phone numbers in the _with_phone workbooks
Matched each arrived student against Scholarship 7-8-9 (4).xlsx by
surname and given name (both must clear a 0.80 similarity threshold,
with Cyrillic transliterated and Uzbek Latin spelling variants folded)
so near-namesakes are left blank rather than mismatched.

Phones normalised to the local 9-digit form; the 998 country code and
stray grade digits in the source cells are stripped.

Filled: 49/53 (grade 7), 52/54 (grade 8), 52/54 (grade 9).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Do3Td8B6ipcHRjUPD7AL1W
</commit_message>
<xml_diff>
--- a/QABUL_IMTIHONI_7-SINF_with_phone.xlsx
+++ b/QABUL_IMTIHONI_7-SINF_with_phone.xlsx
@@ -236,7 +236,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -285,6 +285,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -803,7 +806,11 @@
       </c>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="18" t="n"/>
-      <c r="Q6" s="4" t="n"/>
+      <c r="Q6" s="20" t="inlineStr">
+        <is>
+          <t>977769304</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -855,7 +862,11 @@
       </c>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="18" t="n"/>
-      <c r="Q7" s="4" t="n"/>
+      <c r="Q7" s="20" t="inlineStr">
+        <is>
+          <t>931187404</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -907,7 +918,11 @@
       </c>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="18" t="n"/>
-      <c r="Q8" s="4" t="n"/>
+      <c r="Q8" s="20" t="inlineStr">
+        <is>
+          <t>934260980</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -959,7 +974,11 @@
       </c>
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="18" t="n"/>
-      <c r="Q9" s="4" t="n"/>
+      <c r="Q9" s="20" t="inlineStr">
+        <is>
+          <t>907718449</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1011,7 +1030,11 @@
       </c>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="18" t="n"/>
-      <c r="Q10" s="4" t="n"/>
+      <c r="Q10" s="20" t="inlineStr">
+        <is>
+          <t>950223035</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1063,7 +1086,11 @@
       </c>
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="18" t="n"/>
-      <c r="Q11" s="4" t="n"/>
+      <c r="Q11" s="20" t="inlineStr">
+        <is>
+          <t>998800476</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1167,7 +1194,11 @@
       </c>
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="18" t="n"/>
-      <c r="Q13" s="4" t="n"/>
+      <c r="Q13" s="20" t="inlineStr">
+        <is>
+          <t>905830099</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1219,7 +1250,11 @@
       </c>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="18" t="n"/>
-      <c r="Q14" s="4" t="n"/>
+      <c r="Q14" s="20" t="inlineStr">
+        <is>
+          <t>935450845</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1271,7 +1306,11 @@
       </c>
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="18" t="n"/>
-      <c r="Q15" s="4" t="n"/>
+      <c r="Q15" s="20" t="inlineStr">
+        <is>
+          <t>990248855</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1323,7 +1362,11 @@
       </c>
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="18" t="n"/>
-      <c r="Q16" s="4" t="n"/>
+      <c r="Q16" s="20" t="inlineStr">
+        <is>
+          <t>910163363</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1375,7 +1418,11 @@
       </c>
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="18" t="n"/>
-      <c r="Q17" s="4" t="n"/>
+      <c r="Q17" s="20" t="inlineStr">
+        <is>
+          <t>946001681</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1427,7 +1474,11 @@
       </c>
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="18" t="n"/>
-      <c r="Q18" s="4" t="n"/>
+      <c r="Q18" s="20" t="inlineStr">
+        <is>
+          <t>997752136</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1479,7 +1530,11 @@
       </c>
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="18" t="n"/>
-      <c r="Q19" s="4" t="n"/>
+      <c r="Q19" s="20" t="inlineStr">
+        <is>
+          <t>999880504</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1531,7 +1586,11 @@
       </c>
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="18" t="n"/>
-      <c r="Q20" s="4" t="n"/>
+      <c r="Q20" s="20" t="inlineStr">
+        <is>
+          <t>997865886</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1583,7 +1642,11 @@
       </c>
       <c r="O21" s="5" t="n"/>
       <c r="P21" s="18" t="n"/>
-      <c r="Q21" s="4" t="n"/>
+      <c r="Q21" s="20" t="inlineStr">
+        <is>
+          <t>909505631</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1635,7 +1698,11 @@
       </c>
       <c r="O22" s="5" t="n"/>
       <c r="P22" s="18" t="n"/>
-      <c r="Q22" s="4" t="n"/>
+      <c r="Q22" s="20" t="inlineStr">
+        <is>
+          <t>946161485</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1687,7 +1754,11 @@
       </c>
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="18" t="n"/>
-      <c r="Q23" s="4" t="n"/>
+      <c r="Q23" s="20" t="inlineStr">
+        <is>
+          <t>911621772</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1739,7 +1810,11 @@
       </c>
       <c r="O24" s="5" t="n"/>
       <c r="P24" s="18" t="n"/>
-      <c r="Q24" s="4" t="n"/>
+      <c r="Q24" s="20" t="inlineStr">
+        <is>
+          <t>977450315</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1791,7 +1866,11 @@
       </c>
       <c r="O25" s="5" t="n"/>
       <c r="P25" s="18" t="n"/>
-      <c r="Q25" s="4" t="n"/>
+      <c r="Q25" s="20" t="inlineStr">
+        <is>
+          <t>908671988</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1843,7 +1922,11 @@
       </c>
       <c r="O26" s="5" t="n"/>
       <c r="P26" s="18" t="n"/>
-      <c r="Q26" s="4" t="n"/>
+      <c r="Q26" s="20" t="inlineStr">
+        <is>
+          <t>935488091</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1895,7 +1978,11 @@
       </c>
       <c r="O27" s="5" t="n"/>
       <c r="P27" s="18" t="n"/>
-      <c r="Q27" s="4" t="n"/>
+      <c r="Q27" s="20" t="inlineStr">
+        <is>
+          <t>998478877</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1947,7 +2034,11 @@
       </c>
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="18" t="n"/>
-      <c r="Q28" s="4" t="n"/>
+      <c r="Q28" s="20" t="inlineStr">
+        <is>
+          <t>909113133</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1999,7 +2090,11 @@
       </c>
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="18" t="n"/>
-      <c r="Q29" s="4" t="n"/>
+      <c r="Q29" s="20" t="inlineStr">
+        <is>
+          <t>950858090</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2051,7 +2146,11 @@
       </c>
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="18" t="n"/>
-      <c r="Q30" s="4" t="n"/>
+      <c r="Q30" s="20" t="inlineStr">
+        <is>
+          <t>977503433</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2103,7 +2202,11 @@
       </c>
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="18" t="n"/>
-      <c r="Q31" s="4" t="n"/>
+      <c r="Q31" s="20" t="inlineStr">
+        <is>
+          <t>977030079</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2155,7 +2258,11 @@
       </c>
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="18" t="n"/>
-      <c r="Q32" s="4" t="n"/>
+      <c r="Q32" s="20" t="inlineStr">
+        <is>
+          <t>977004435</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2207,7 +2314,11 @@
       </c>
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="18" t="n"/>
-      <c r="Q33" s="4" t="n"/>
+      <c r="Q33" s="20" t="inlineStr">
+        <is>
+          <t>983331041</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2259,7 +2370,11 @@
       </c>
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="18" t="n"/>
-      <c r="Q34" s="4" t="n"/>
+      <c r="Q34" s="20" t="inlineStr">
+        <is>
+          <t>900374634</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2311,7 +2426,11 @@
       </c>
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="18" t="n"/>
-      <c r="Q35" s="4" t="n"/>
+      <c r="Q35" s="20" t="inlineStr">
+        <is>
+          <t>935420079</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2363,7 +2482,11 @@
       </c>
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="18" t="n"/>
-      <c r="Q36" s="4" t="n"/>
+      <c r="Q36" s="20" t="inlineStr">
+        <is>
+          <t>943815991</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2415,7 +2538,11 @@
       </c>
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="18" t="n"/>
-      <c r="Q37" s="4" t="n"/>
+      <c r="Q37" s="20" t="inlineStr">
+        <is>
+          <t>995318591</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2467,7 +2594,11 @@
       </c>
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="18" t="n"/>
-      <c r="Q38" s="4" t="n"/>
+      <c r="Q38" s="20" t="inlineStr">
+        <is>
+          <t>884248088</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2519,7 +2650,11 @@
       </c>
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="18" t="n"/>
-      <c r="Q39" s="4" t="n"/>
+      <c r="Q39" s="20" t="inlineStr">
+        <is>
+          <t>903230646</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2571,7 +2706,11 @@
       </c>
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="18" t="n"/>
-      <c r="Q40" s="4" t="n"/>
+      <c r="Q40" s="20" t="inlineStr">
+        <is>
+          <t>955010808</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -2623,7 +2762,11 @@
       </c>
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="18" t="n"/>
-      <c r="Q41" s="4" t="n"/>
+      <c r="Q41" s="20" t="inlineStr">
+        <is>
+          <t>977770480</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -2675,7 +2818,7 @@
       </c>
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="18" t="n"/>
-      <c r="Q42" s="4" t="inlineStr">
+      <c r="Q42" s="20" t="inlineStr">
         <is>
           <t>946653461</t>
         </is>
@@ -2783,7 +2926,7 @@
       </c>
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="18" t="n"/>
-      <c r="Q44" s="4" t="inlineStr">
+      <c r="Q44" s="20" t="inlineStr">
         <is>
           <t>333304334</t>
         </is>
@@ -2891,7 +3034,7 @@
       </c>
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="18" t="n"/>
-      <c r="Q46" s="4" t="inlineStr">
+      <c r="Q46" s="20" t="inlineStr">
         <is>
           <t>973270345</t>
         </is>
@@ -2947,7 +3090,7 @@
       </c>
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="18" t="n"/>
-      <c r="Q47" s="4" t="inlineStr">
+      <c r="Q47" s="20" t="inlineStr">
         <is>
           <t>981296404</t>
         </is>
@@ -3003,7 +3146,11 @@
       </c>
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="18" t="n"/>
-      <c r="Q48" s="4" t="n"/>
+      <c r="Q48" s="20" t="inlineStr">
+        <is>
+          <t>911296404</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -3055,7 +3202,7 @@
       </c>
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="18" t="n"/>
-      <c r="Q49" s="4" t="inlineStr">
+      <c r="Q49" s="20" t="inlineStr">
         <is>
           <t>935941727</t>
         </is>
@@ -3111,7 +3258,7 @@
       </c>
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="18" t="n"/>
-      <c r="Q50" s="4" t="inlineStr">
+      <c r="Q50" s="20" t="inlineStr">
         <is>
           <t>909188700</t>
         </is>
@@ -3167,7 +3314,7 @@
       </c>
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="18" t="n"/>
-      <c r="Q51" s="4" t="inlineStr">
+      <c r="Q51" s="20" t="inlineStr">
         <is>
           <t>236465959</t>
         </is>
@@ -3223,7 +3370,7 @@
       </c>
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="18" t="n"/>
-      <c r="Q52" s="4" t="inlineStr">
+      <c r="Q52" s="20" t="inlineStr">
         <is>
           <t>935085869</t>
         </is>
@@ -3279,7 +3426,7 @@
       </c>
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="18" t="n"/>
-      <c r="Q53" s="4" t="inlineStr">
+      <c r="Q53" s="20" t="inlineStr">
         <is>
           <t>950140207</t>
         </is>
@@ -3335,7 +3482,7 @@
       </c>
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="18" t="n"/>
-      <c r="Q54" s="4" t="inlineStr">
+      <c r="Q54" s="20" t="inlineStr">
         <is>
           <t>930065445</t>
         </is>
@@ -3391,7 +3538,7 @@
       </c>
       <c r="O55" s="5" t="n"/>
       <c r="P55" s="18" t="n"/>
-      <c r="Q55" s="4" t="inlineStr">
+      <c r="Q55" s="20" t="inlineStr">
         <is>
           <t>930075429</t>
         </is>
@@ -3447,7 +3594,7 @@
       </c>
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="18" t="n"/>
-      <c r="Q56" s="4" t="inlineStr">
+      <c r="Q56" s="20" t="inlineStr">
         <is>
           <t>970040565</t>
         </is>
@@ -3503,7 +3650,7 @@
       </c>
       <c r="O57" s="5" t="n"/>
       <c r="P57" s="18" t="n"/>
-      <c r="Q57" s="4" t="inlineStr">
+      <c r="Q57" s="20" t="inlineStr">
         <is>
           <t>935884941</t>
         </is>

</xml_diff>